<commit_message>
criando e melhorando o sincronizador de pastas e dados de clientes
</commit_message>
<xml_diff>
--- a/foton_system/foton_make/testes/base.xlsx
+++ b/foton_system/foton_make/testes/base.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/893df2c86f46c70e/LAMP ARQUITETURA/foton/foton_system/foton_make/testes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{AFF7D401-F903-4095-A4BF-F17281F15F13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65C7F3B8-BE5C-4157-BF5D-CCC7AA8396A0}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{AFF7D401-F903-4095-A4BF-F17281F15F13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9694861A-0C88-45C9-8185-0103A2F54954}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="28800" windowHeight="11295" activeTab="1" xr2:uid="{BFD264AB-D9E2-40EC-8F40-C24696CBF67A}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="23565" windowHeight="11295" xr2:uid="{BFD264AB-D9E2-40EC-8F40-C24696CBF67A}"/>
   </bookViews>
   <sheets>
     <sheet name="baseClientes" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
   <si>
     <t>NomeCliente</t>
   </si>
@@ -79,6 +79,15 @@
   </si>
   <si>
     <t>CodCliente</t>
+  </si>
+  <si>
+    <t>Alias</t>
+  </si>
+  <si>
+    <t>LUCAS LAMP</t>
+  </si>
+  <si>
+    <t>PROJ-1</t>
   </si>
 </sst>
 </file>
@@ -149,6 +158,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -468,17 +481,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EA0F879-0B59-4EC3-A645-64CCE49FFB13}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="1"/>
+    <col min="3" max="3" width="15.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -486,23 +500,29 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="1">
         <v>3999354100</v>
       </c>
-      <c r="D2" s="1">
+      <c r="E2" s="1">
         <v>20051994</v>
       </c>
     </row>
@@ -513,19 +533,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93B3DC20-42E1-4C8A-8773-DD4FD855472F}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="4" max="4" width="14.28515625" style="1" customWidth="1"/>
+    <col min="5" max="6" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -536,19 +557,22 @@
         <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -558,16 +582,19 @@
       <c r="C2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="2">
         <v>1042024</v>
       </c>
-      <c r="E2" s="1">
+      <c r="F2" s="1">
         <v>2500</v>
       </c>
-      <c r="F2" s="1">
+      <c r="G2" s="1">
         <v>5000</v>
       </c>
-      <c r="G2" s="1">
+      <c r="H2" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>